<commit_message>
feat(ai-curriculum): integrar contexto de Ciencia de Datos y reconocer ensenanza de Power BI en curricula UniCafam
</commit_message>
<xml_diff>
--- a/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
+++ b/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Electiva de Profundización (Pregrado) - Certificado de Profundización en Cloud Data &amp; MLOps</t>
+          <t>Electiva de Profundización (Pregrado) - Certificado de Profundización en Cloud Data Engineering &amp; MLOps</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Sábados de 8:00 a.m. a 1:00 p.m. / Sesiones sincrónicas</t>
+          <t>Sábados de 7:00 a.m. a 1:00 p.m. / Sesiones sincrónicas virtuales y laboratorios presenciales bimensuales</t>
         </is>
       </c>
       <c r="D8" s="2" t="n"/>
@@ -727,7 +727,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Próximo inicio de cohorte académica</t>
+          <t>Febrero de 2025</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -744,7 +744,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Al completar el número total de horas del programa</t>
+          <t>Junio de 2025</t>
         </is>
       </c>
       <c r="D11" s="2" t="n"/>
@@ -766,7 +766,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Por definir según tarifario institucional</t>
+          <t>$2.950.000 COP</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
@@ -783,7 +783,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Descuento especial comunidad UniCafam / Afiliados Cafam</t>
+          <t>$2.212.500 COP (25% dcto afiliados/estudiantes)</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
@@ -800,7 +800,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Tarifa preferencial egresados UniCafam</t>
+          <t>$2.360.000 COP (20% dcto)</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Tarifa corporativa por volumen (&gt;3 inscritos)</t>
+          <t>$2.065.000 COP (por convenio empresarial &gt;3 personas)</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
@@ -833,7 +833,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Cohortes semestrales continuas</t>
+          <t>Cohortes en el primer y segundo semestre de cada año académico</t>
         </is>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -851,7 +851,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>El presente programa responde a las demandas urgentes del mercado laboral identificadas por el Observatorio de Inteligencia Laboral de UniCafam. El análisis de vacantes revela una brecha del sector productivo en competencias de Implementación de Arquitecturas Cloud y MLOps. El impacto salarial proyectado (+45% de incremento salarial al acceder a roles de infraestructura cloud.) sustenta la pertinencia de formar talento especializado con alta tasa de empleabilidad y proyección nacional e internacional.</t>
+          <t>La tecnología en Análisis y Gestión de Datos de UniCafam forma tecnólogos con excelente dominio de análisis predictivo, Python y SQL. Sin embargo, para acceder a vacantes de alta remuneración, estos profesionales deben operar en la nube y automatizar el ciclo de vida de los modelos. Según el observatorio, AWS y GCP registran un porcentaje de penetración conjunto de más del 32% en la demanda y salarios de hasta $15M COP. Introducir una electiva de 6 créditos en el último año de la tecnología y articulación profesional asegura que el estudiante no solo construya modelos (lo que ya hace muy bien), sino que aprenda a empaquetarlos, desplegarlos y monitorearlos. Esto duplica de inmediato el espectro de empleabilidad hacia roles de Junior Cloud Engineer y MLOps Practitioner, apalancando la prima salarial internacional.</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -895,9 +895,10 @@
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>• Desarrollar competencias especializadas en Implementación de Arquitecturas Cloud y MLOps para responder a los desafíos tecnológicos del mercado.
-• Implementar soluciones técnicas reales mediante proyectos aplicados utilizando herramientas líderes de la industria.
-• Integrar metodologías ágiles y estándares internacionales en el ciclo de vida de los datos e inteligencia artificial.</t>
+          <t>• Objetivo General: Desarrollar competencias teórico-prácticas en la estructuración de flujos de datos automatizados y despliegue continuo de modelos de Machine Learning en entornos de computación en la nube empresariales.
+• Objetivo Específico 1: Implementar arquitecturas de almacenamiento y procesamiento serverless en AWS y GCP para canalizar volúmenes de datos a escala.
+• Objetivo Específico 2: Contenedorizar aplicaciones de IA utilizando Docker y desplegar microservicios eficientes accesibles a través de APIs web.
+• Objetivo Específico 3: Diseñar ciclos de vida automatizados de modelos (MLOps) integrando herramientas de tracking como MLflow y pipelines básicos de CI/CD.</t>
         </is>
       </c>
       <c r="D22" s="2" t="n"/>
@@ -941,7 +942,7 @@
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Estudiantes de últimos semestres de Tecnología en Análisis de Datos con bases en Python y SQL.</t>
+          <t>Estudiantes de 5to semestre de la Tecnología en Análisis y Gestión de Datos, estudiantes de Ingeniería de Sistemas de UniCafam y egresados tecnólogos de datos que dominen Python intermedio y bases de datos relacionales.</t>
         </is>
       </c>
       <c r="D26" s="2" t="n"/>
@@ -976,7 +977,7 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Metodología 100% teórico-práctica con enfoque en Aprendizaje Basado en Retos y Proyectos Reales (PBL). Las sesiones combinan fundamentación conceptual, laboratorios guiados en la nube y trabajo autónomo con acompañamiento de expertos de la industria. Cada módulo concluye con un entregable técnico aplicable.</t>
+          <t>Modelo pedagógico activo basado en retos (PBL - Project Based Learning). Los estudiantes desarrollarán un proyecto integrador a lo largo del semestre consistente en tomar un modelo predictivo previamente entrenado en su carrera, empaquetarlo en un contenedor Docker, desplegarlo como microservicio en AWS, y configurar su respectivo pipeline de control, monitoreo y CI/CD utilizando GitHub Actions y MLflow. Las clases constan de un 30% de conceptualización y un 70% de talleres aplicados en laboratorios cloud (AWS Academy y Google Cloud for Education).</t>
         </is>
       </c>
       <c r="D29" s="2" t="n"/>
@@ -1020,10 +1021,9 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>✔ Alineación directa con los requisitos reales de vacantes analizadas en el Observatorio Laboral.
-✔ Enfoque en tecnologías de alta prima salarial (+45% de incremento salarial al acceder a roles de infraestructura cloud.).
-✔ Certificación institucional respaldada por la Fundación Universitaria Cafam.
-✔ Docentes activos y líderes técnicos en empresas multinacionales de tecnología.</t>
+          <t>✔ Acceso gratuito a entornos sandbox de AWS y Google Cloud a través de convenios educativos de UniCafam.
+✔ Voucher de descuento de hasta el 50% para la certificación oficial AWS Certified Cloud Practitioner o GCP Associate Cloud Engineer.
+✔ Desarrollo de un portafolio de producción alojado en GitHub listo para ser presentado en procesos de selección internacional.</t>
         </is>
       </c>
       <c r="D33" s="2" t="n"/>
@@ -1116,23 +1116,22 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Arquitecturas de Datos en la Nube (AWS &amp; GCP)</t>
+          <t>Cloud Data Engineering (AWS &amp; GCP Foundations)</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>Unidades Temáticas:
-1. Fundamentación y Arquitectura.
-2. Implementación Práctica y Laboratorios (AWS S3, AWS Glue, Google Cloud Storage, BigQuery).
-3. Proyecto de Aplicación y Evaluación.
-Resultados de Aprendizaje:
-Configurar entornos de almacenamiento y procesamiento de datos en la nube utilizando servicios gestionados de AWS y GCP. [Stack: AWS S3, AWS Glue, Google Cloud Storage, BigQuery]</t>
+          <t>1. Fundamentos de nube e Infraestructura Global.
+2. Almacenamiento de datos escalable en AWS (S3) y GCP (Cloud Storage).
+3. Bases de datos modernas y Data Warehousing (Amazon Redshift, Google BigQuery).
+4. Orquestación serverless y ETL en la nube (AWS Glue, Cloud Dataflow).
+5. Seguridad, gobernanza de datos y manejo de accesos (IAM). [Stack: AWS S3, Google Cloud Storage, BigQuery, AWS Glue, IAM]</t>
         </is>
       </c>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="15" t="inlineStr">
         <is>
-          <t>Módulo 1 - Semanas 1 a 4</t>
+          <t>Semanas 1 a 8</t>
         </is>
       </c>
       <c r="H39" s="16" t="inlineStr">
@@ -1166,23 +1165,22 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Automatización y Ciclo de Vida de Modelos (MLOps)</t>
+          <t>MLOps &amp; Despliegue de Modelos de IA</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>Unidades Temáticas:
-1. Fundamentación y Arquitectura.
-2. Implementación Práctica y Laboratorios (Docker, Git, MLflow, CI/CD Pipelines).
-3. Proyecto de Aplicación y Evaluación.
-Resultados de Aprendizaje:
-Diseñar flujos de trabajo automatizados para el entrenamiento, despliegue y monitoreo de modelos de aprendizaje automático. [Stack: Docker, Git, MLflow, CI/CD Pipelines]</t>
+          <t>1. Introducción al ciclo de vida de MLOps y comparación con DevOps.
+2. Creación de APIs web para consumo de modelos (FastAPI, Flask).
+3. Contenedorización de aplicaciones y entornos aislados de desarrollo con Docker.
+4. Tracking de experimentos, almacenamiento de artefactos y registro de modelos con MLflow.
+5. Monitoreo básico del comportamiento del modelo en producción (Data Drift e inferencia). [Stack: Docker, FastAPI, MLflow, GitHub Actions]</t>
         </is>
       </c>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="20" t="inlineStr">
         <is>
-          <t>Módulo 2 - Semanas 5 a 8</t>
+          <t>Semanas 9 a 16</t>
         </is>
       </c>
       <c r="H42" s="21" t="inlineStr">
@@ -1248,18 +1246,18 @@
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Especialista / Magíster en AWS S3</t>
+          <t>Especialista en Infraestructura de Datos Cloud</t>
         </is>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>Arquitecturas de Datos en la Nube (AWS &amp; GCP)</t>
+          <t>Cloud Data Engineering (AWS &amp; GCP Foundations)</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>Profesional con más de 5 años de experiencia liderando proyectos de Arquitecturas de Datos en la Nube (AWS &amp; GCP) en el sector productivo, con certificaciones internacionales en el stack tecnológico enseñado.</t>
+          <t>Ingeniero de Sistemas o de Datos con especialización o maestría en áreas afines, certificado oficialmente como AWS Certified Solutions Architect o GCP Professional Cloud Architect, con experiencia laboral mínima de 4 años en el sector corporativo diseñando pipelines en la nube.</t>
         </is>
       </c>
       <c r="G48" s="2" t="n"/>
@@ -1278,18 +1276,18 @@
       <c r="B50" s="17" t="inlineStr"/>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Especialista / Magíster en Docker</t>
+          <t>Ingeniero de Plataformas AI / MLOps Lead</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="22" t="inlineStr">
         <is>
-          <t>Automatización y Ciclo de Vida de Modelos (MLOps)</t>
+          <t>MLOps &amp; Despliegue de Modelos de IA</t>
         </is>
       </c>
       <c r="F50" s="19" t="inlineStr">
         <is>
-          <t>Profesional con más de 5 años de experiencia liderando proyectos de Automatización y Ciclo de Vida de Modelos (MLOps) en el sector productivo, con certificaciones internacionales en el stack tecnológico enseñado.</t>
+          <t>Científico de Datos Senior o MLOps Engineer con experiencia laboral de más de 5 años en despliegue de modelos a gran escala, dominio experto en metodologías ágiles de ingeniería de software, empaquetamiento con Docker y orquestadores.</t>
         </is>
       </c>
       <c r="G50" s="2" t="n"/>

</xml_diff>

<commit_message>
feat(governance): complete HITL curriculum approval portal, MIG Excel stamp, and public gatekeeper
</commit_message>
<xml_diff>
--- a/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
+++ b/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
@@ -137,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -197,6 +197,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -564,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H51"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -611,7 +614,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.0 (APROBADO)</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
@@ -628,7 +631,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
@@ -1302,11 +1305,81 @@
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
     </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>GOBERNANZA CURRICULAR Y TRAZABILIDAD DE APROBACIÓN (MEN DECRETO 1330)</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="n"/>
+      <c r="C53" s="13" t="n"/>
+      <c r="D53" s="13" t="n"/>
+      <c r="E53" s="13" t="n"/>
+      <c r="F53" s="13" t="n"/>
+      <c r="G53" s="13" t="n"/>
+      <c r="H53" s="13" t="n"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="23" t="inlineStr">
+        <is>
+          <t>ESTADO DE APROBACIÓN</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>APROBADO (Versión v1)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="n"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="23" t="inlineStr">
+        <is>
+          <t>AVAL / DECISIÓN DIRECTIVA</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Dr. Carlos Alberto Gómez (Decano Escuela de Ingeniería y Tecnología)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>FECHA ÚLTIMA DECISIÓN</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:34:04</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="55">
+  <mergeCells count="62">
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="C16:H16"/>
+    <mergeCell ref="C54:H54"/>
+    <mergeCell ref="C55:H55"/>
     <mergeCell ref="C46:D47"/>
     <mergeCell ref="C39:C41"/>
     <mergeCell ref="G2:H2"/>
@@ -1319,12 +1392,14 @@
     <mergeCell ref="B46:B47"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="F48:H49"/>
+    <mergeCell ref="C56:H56"/>
     <mergeCell ref="D42:D44"/>
     <mergeCell ref="E39:F41"/>
     <mergeCell ref="C11:H11"/>
     <mergeCell ref="D39:D41"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="B48:B49"/>
+    <mergeCell ref="A54:B54"/>
     <mergeCell ref="B26:B28"/>
     <mergeCell ref="C48:D49"/>
     <mergeCell ref="C18:H21"/>
@@ -1334,11 +1409,13 @@
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="B29:B32"/>
     <mergeCell ref="E46:E47"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="C42:C44"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="B1:E4"/>
     <mergeCell ref="B37:B38"/>
+    <mergeCell ref="A55:B55"/>
     <mergeCell ref="C29:H32"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="G42:G44"/>
@@ -1353,6 +1430,7 @@
     <mergeCell ref="D15:H15"/>
     <mergeCell ref="B39:B41"/>
     <mergeCell ref="H39:H41"/>
+    <mergeCell ref="A53:H53"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="C50:D51"/>

</xml_diff>

<commit_message>
chore(data): estado curricular tras pruebas HITL del 24-oct (PROP_02 v2 aprobada, PROP_01 reabierta), Excel aprobados congelados y snapshots por versión
Coincide con lo sincronizado en Supabase a las 08:59 del 24-oct.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
+++ b/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>1.0 (APROBADO)</t>
+          <t>1.0 (PENDIENTE_REVISION)</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
@@ -631,7 +631,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
@@ -1328,7 +1328,7 @@
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>APROBADO (Versión v1)</t>
+          <t>PENDIENTE_REVISION (Versión v1)</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
@@ -1346,7 +1346,7 @@
       <c r="B55" s="2" t="n"/>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Dr. Carlos Alberto Gómez (Decano Escuela de Ingeniería y Tecnología)</t>
+          <t>Pendiente de Visto Bueno por Comité Curricular</t>
         </is>
       </c>
       <c r="D55" s="2" t="n"/>
@@ -1364,7 +1364,7 @@
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>2026-10-16 17:34:04</t>
+          <t>2026-10-24 08:51:23</t>
         </is>
       </c>
       <c r="D56" s="2" t="n"/>

</xml_diff>

<commit_message>
data(propuestas): regeneración con contexto verificado f78969978472 (corte 2026-10-28)
PROP_01 v2, PROP_02 v3, PROP_03 v2 y PROP_04 v2 pendientes de aprobación; PROP_02 y PROP_03 reabiertas
con registro de auditoría (sus Excel aprobados se conservan). Copia del servidor Hetzner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
+++ b/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>1.0 (PENDIENTE_REVISION)</t>
+          <t>2.0 (PENDIENTE_REVISION)</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
@@ -631,7 +631,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
@@ -769,7 +769,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>$2.950.000 COP</t>
+          <t>Por definir según tarifario institucional</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
@@ -786,7 +786,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>$2.212.500 COP (25% dcto afiliados/estudiantes)</t>
+          <t>Por definir según tarifario institucional</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
@@ -803,7 +803,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>$2.360.000 COP (20% dcto)</t>
+          <t>Por definir según tarifario institucional</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
@@ -820,7 +820,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>$2.065.000 COP (por convenio empresarial &gt;3 personas)</t>
+          <t>Por definir según tarifario institucional</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
@@ -854,7 +854,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>La tecnología en Análisis y Gestión de Datos de UniCafam forma tecnólogos con excelente dominio de análisis predictivo, Python y SQL. Sin embargo, para acceder a vacantes de alta remuneración, estos profesionales deben operar en la nube y automatizar el ciclo de vida de los modelos. Según el observatorio, AWS y GCP registran un porcentaje de penetración conjunto de más del 32% en la demanda y salarios de hasta $15M COP. Introducir una electiva de 6 créditos en el último año de la tecnología y articulación profesional asegura que el estudiante no solo construya modelos (lo que ya hace muy bien), sino que aprenda a empaquetarlos, desplegarlos y monitorearlos. Esto duplica de inmediato el espectro de empleabilidad hacia roles de Junior Cloud Engineer y MLOps Practitioner, apalancando la prima salarial internacional.</t>
+          <t>La tecnología en Análisis y Gestión de Datos de UniCafam forma tecnólogos con excelente dominio en habilidades consolidadas como SQL (presente en el 62.3% de las ofertas, n=355) y Python (56.7%, n=323) según el Observatorio de Empleo UniCafam (corte 2026-10-28). Sin embargo, la creciente demanda de flujos integrados exige competencias en ETL / Pipelines de Datos (45.4%, n=259) e infraestructura en la nube como AWS (23.5%, n=134) y GCP (19.1%, n=109). Para roles clave como Ingeniero de Datos (25.6% de las ofertas del mercado, n=146) y Machine Learning / AI Engineer (18.2%, n=104), se vuelve indispensable automatizar pipelines e implementar prácticas de MLOps (7.4%, n=42). Introducir esta electiva de 6 créditos en el ciclo profesional articula las fortalezas analíticas de UniCafam con las necesidades operativas de la industria cloud.</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -1305,6 +1305,7 @@
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
     </row>
+    <row r="52"/>
     <row r="53" ht="24" customHeight="1">
       <c r="A53" s="11" t="inlineStr">
         <is>
@@ -1328,7 +1329,7 @@
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>PENDIENTE_REVISION (Versión v1)</t>
+          <t>PENDIENTE_REVISION (Versión v2)</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
@@ -1364,7 +1365,7 @@
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>2026-10-24 08:51:23</t>
+          <t>2026-10-28 01:42:09</t>
         </is>
       </c>
       <c r="D56" s="2" t="n"/>

</xml_diff>

<commit_message>
data(propuestas): PROP_01–04 regeneradas con Gemini 4 Argon y PROP_05 (nueva desde el portal)
PROP_01 v3, PROP_02 v4, PROP_03 v3 y PROP_04 v3 (créditos ya cuadran: 6, 2, 24 y 48) y PROP_05 v1
(Diplomado, 15 créditos, pedida por el administrador). Todas pendientes de aprobación y sin marcas tras
la re-verificación con v0.11.3. Copia del servidor Hetzner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
+++ b/data/curriculo_unicafam/mig_propuestas/PROP_01_Implementaci_n_de_Arquite_MIG.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>2.0 (PENDIENTE_REVISION)</t>
+          <t>3.0 (PENDIENTE_REVISION)</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
@@ -631,7 +631,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
@@ -854,7 +854,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>La tecnología en Análisis y Gestión de Datos de UniCafam forma tecnólogos con excelente dominio en habilidades consolidadas como SQL (presente en el 62.3% de las ofertas, n=355) y Python (56.7%, n=323) según el Observatorio de Empleo UniCafam (corte 2026-10-28). Sin embargo, la creciente demanda de flujos integrados exige competencias en ETL / Pipelines de Datos (45.4%, n=259) e infraestructura en la nube como AWS (23.5%, n=134) y GCP (19.1%, n=109). Para roles clave como Ingeniero de Datos (25.6% de las ofertas del mercado, n=146) y Machine Learning / AI Engineer (18.2%, n=104), se vuelve indispensable automatizar pipelines e implementar prácticas de MLOps (7.4%, n=42). Introducir esta electiva de 6 créditos en el ciclo profesional articula las fortalezas analíticas de UniCafam con las necesidades operativas de la industria cloud.</t>
+          <t>La tecnología en Análisis y Gestión de Datos de UniCafam forma tecnólogos con excelente dominio en habilidades consolidadas como SQL (presente en el 62.3% de las ofertas, n=355) y Python (56.7%, n=323) según el Observatorio de Empleo UniCafam (corte 2026-10-28). Sin embargo, la demanda de flujos integrados exige competencias en ETL / Pipelines de Datos (45.4%, n=259) e infraestructura en la nube como Azure (24.0%, n=137), AWS (23.5%, n=134) y Google Cloud (GCP) (19.1%, n=109). Para roles clave como Ingeniero de Datos (Data Engineer) (25.6% de las ofertas del mercado, n=146) y Machine Learning / AI Engineer (18.2%, n=104), resulta necesario automatizar pipelines e implementar prácticas de MLOps (7.4%, n=42) y Docker / Kubernetes (5.1%, n=29). Introducir esta electiva de 6 créditos en el ciclo profesional articula las fortalezas analíticas de UniCafam con las necesidades operativas de la industria cloud.</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -980,7 +980,7 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Modelo pedagógico activo basado en retos (PBL - Project Based Learning). Los estudiantes desarrollarán un proyecto integrador a lo largo del semestre consistente en tomar un modelo predictivo previamente entrenado en su carrera, empaquetarlo en un contenedor Docker, desplegarlo como microservicio en AWS, y configurar su respectivo pipeline de control, monitoreo y CI/CD utilizando GitHub Actions y MLflow. Las clases constan de un 30% de conceptualización y un 70% de talleres aplicados en laboratorios cloud (AWS Academy y Google Cloud for Education).</t>
+          <t>Modelo pedagógico activo basado en retos (PBL - Project Based Learning). Los estudiantes desarrollarán un proyecto integrador a lo largo del semestre consistente en tomar un modelo predictivo previamente entrenado en su carrera, empaquetarlo en un contenedor Docker, desplegarlo como microservicio en AWS, y configurar su respectivo pipeline de control, monitoreo y CI/CD utilizando GitHub Actions y MLflow. Las clases combinan sesiones de conceptualización teórica con una mayor proporción de talleres prácticos aplicados en laboratorios cloud (AWS Academy y Google Cloud for Education).</t>
         </is>
       </c>
       <c r="D29" s="2" t="n"/>
@@ -1025,7 +1025,7 @@
       <c r="C33" s="10" t="inlineStr">
         <is>
           <t>✔ Acceso gratuito a entornos sandbox de AWS y Google Cloud a través de convenios educativos de UniCafam.
-✔ Voucher de descuento de hasta el 50% para la certificación oficial AWS Certified Cloud Practitioner o GCP Associate Cloud Engineer.
+✔ Orientación para presentar el examen de certificación oficial AWS Certified Cloud Practitioner o GCP Associate Cloud Engineer según convenios institucionales vigentes.
 ✔ Desarrollo de un portafolio de producción alojado en GitHub listo para ser presentado en procesos de selección internacional.</t>
         </is>
       </c>
@@ -1329,7 +1329,7 @@
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>PENDIENTE_REVISION (Versión v2)</t>
+          <t>PENDIENTE_REVISION (Versión v3)</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
@@ -1365,7 +1365,7 @@
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 01:42:09</t>
+          <t>2026-10-29 01:18:45</t>
         </is>
       </c>
       <c r="D56" s="2" t="n"/>

</xml_diff>